<commit_message>
Add TALENTO and BIENESTAR modules with dynamic Excel data; fix Personal KPIs and case sensitivity
</commit_message>
<xml_diff>
--- a/Plantilla_Summar_DEMO.xlsx
+++ b/Plantilla_Summar_DEMO.xlsx
@@ -17,6 +17,8 @@
     <sheet name="ENTREVISTAS_RETIRO" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="SINIESTRO" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="FUEROS_SALUD" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="TALENTO_DISCIPLINARIO" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="BIENESTAR_ACTIVIDADES" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1759,6 +1761,1453 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Empresa</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>NIT</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>Numdocumento</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>Cargo</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="H1" s="9" t="inlineStr">
+        <is>
+          <t>Motivo</t>
+        </is>
+      </c>
+      <c r="I1" s="9" t="inlineStr">
+        <is>
+          <t>Acción</t>
+        </is>
+      </c>
+      <c r="J1" s="9" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="K1" s="9" t="inlineStr">
+        <is>
+          <t>Observaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Distribuciones Pacífico Ltda</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>900.333.444-2</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Distribuciones Pacífico Ltda</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>108550862</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Ana Martínez</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Almacenista</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2025-04-25</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Daño a equipos</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Llamado de atención escrito</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Archivado</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Sin novedad adicional</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Retail Express Colombia</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>900.555.666-3</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Retail Express Colombia</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>103972270</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Sandra García</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Operario de Producción</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2025-04-26</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Bajo rendimiento</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Llamado de atención verbal</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Sin novedad adicional</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Distribuciones Pacífico Ltda</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>900.333.444-2</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Distribuciones Pacífico Ltda</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>107588427</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Diana Torres</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Inspector</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2025-03-01</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Tardanza reiterada</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Llamado de atención verbal</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>En seguimiento</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Sin novedad adicional</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Distribuciones Pacífico Ltda</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>900.333.444-2</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Distribuciones Pacífico Ltda</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>104815317</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>María Hernández</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Técnico</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2025-03-16</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Incumplimiento de normas</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Llamado de atención escrito</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Archivado</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Sin novedad adicional</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Distribuciones Pacífico Ltda</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>900.333.444-2</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Distribuciones Pacífico Ltda</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>101034214</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Carlos Rodríguez</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Auxiliar Logístico</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2025-02-15</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Daño a equipos</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Suspensión 1 día</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Archivado</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Sin novedad adicional</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>900.111.222-1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>108909806</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Ana Rodríguez</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Operario de Producción</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2025-06-10</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Daño a equipos</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Suspensión 1 día</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Archivado</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Sin novedad adicional</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Distribuciones Pacífico Ltda</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>900.333.444-2</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Distribuciones Pacífico Ltda</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>107781119</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Fabio Martínez</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Técnico</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2025-04-15</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Daño a equipos</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Descargo escrito</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Archivado</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Sin novedad adicional</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Retail Express Colombia</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>900.555.666-3</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Retail Express Colombia</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>101028335</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Luis López</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Operario de Producción</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2025-05-21</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Ausentismo injustificado</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Llamado de atención escrito</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Archivado</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Sin novedad adicional</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>900.111.222-1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>108668553</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>María Torres</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Almacenista</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2025-02-09</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Daño a equipos</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Descargo escrito</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Sin novedad adicional</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>900.111.222-1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>102481086</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Andrés Martínez</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Inspector</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Conducta inapropiada</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Llamado de atención verbal</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>En seguimiento</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Sin novedad adicional</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>900.111.222-1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>107991904</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Ana Sánchez</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Técnico</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2025-06-02</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Ausentismo injustificado</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Suspensión 1 día</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>En seguimiento</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Sin novedad adicional</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Distribuciones Pacífico Ltda</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>900.333.444-2</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Distribuciones Pacífico Ltda</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>101455616</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sandra Torres</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Técnico</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2025-05-07</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Conducta inapropiada</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Plan de mejora</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Sin novedad adicional</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Distribuciones Pacífico Ltda</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>900.333.444-2</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Distribuciones Pacífico Ltda</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>105819543</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Pedro López</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Inspector</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2025-02-24</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Conducta inapropiada</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Llamado de atención verbal</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Archivado</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Sin novedad adicional</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Retail Express Colombia</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>900.555.666-3</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Retail Express Colombia</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>103096863</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Diego Martínez</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Inspector</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2025-03-08</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Tardanza reiterada</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Plan de mejora</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>En seguimiento</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Sin novedad adicional</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Retail Express Colombia</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>900.555.666-3</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Retail Express Colombia</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>108698218</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Luis Martínez</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Operario de Producción</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2025-04-07</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Daño a equipos</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Suspensión 3 días</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Sin novedad adicional</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Empresa</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>NIT</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Actividad</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Impacto</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Observaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>900.111.222-1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Ene</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2025-01-15</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Bienvenida 2025 — Celebración inicio de año</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I2" t="n">
+        <v>82</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Carlos Ruiz</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Actividad completada exitosamente</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>900.111.222-1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2025-02-14</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Día de la Amistad — Integración virtual</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>85</v>
+      </c>
+      <c r="I3" t="n">
+        <v>78</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Ana Torres</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Actividad completada exitosamente</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>900.111.222-1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2025-03-08</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Día de la Mujer — Reconocimiento y charla</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Híbrido</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>63</v>
+      </c>
+      <c r="I4" t="n">
+        <v>71</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Ana Torres</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Actividad completada exitosamente</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>900.111.222-1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Abr</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2025-04-22</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Pausas activas saludables</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>91</v>
+      </c>
+      <c r="I5" t="n">
+        <v>85</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Ana Torres</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Actividad completada exitosamente</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>900.111.222-1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2025-05-15</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Celebración Día de la Madre</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>78</v>
+      </c>
+      <c r="I6" t="n">
+        <v>80</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Laura Gómez</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Actividad completada exitosamente</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>900.111.222-1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2025-05-28</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Taller Bienestar Emocional y Estrés</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>54</v>
+      </c>
+      <c r="I7" t="n">
+        <v>65</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>María López</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Actividad completada exitosamente</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>900.111.222-1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2025-06-05</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Actividad deportiva — Campeonato interno</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>110</v>
+      </c>
+      <c r="I8" t="n">
+        <v>90</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Ana Torres</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Actividad completada exitosamente</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>900.111.222-1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Grupo Industrial Norte S.A.S</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2025-06-20</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Charla nutrición y hábitos saludables</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>67</v>
+      </c>
+      <c r="I9" t="n">
+        <v>74</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Carlos Ruiz</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Actividad completada exitosamente</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2671,8 +4120,6 @@
           <t>2025-06-22</t>
         </is>
       </c>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr">
         <is>
           <t>Conforme</t>
@@ -3103,8 +4550,6 @@
           <t>2025-06-22</t>
         </is>
       </c>
-      <c r="AA9" t="inlineStr"/>
-      <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr">
         <is>
           <t>Conforme</t>
@@ -3666,7 +5111,6 @@
       <c r="W13" t="n">
         <v>8</v>
       </c>
-      <c r="X13" t="inlineStr"/>
       <c r="Y13" t="inlineStr">
         <is>
           <t>Normal</t>
@@ -3677,8 +5121,6 @@
           <t>2025-06-22</t>
         </is>
       </c>
-      <c r="AA13" t="inlineStr"/>
-      <c r="AB13" t="inlineStr"/>
       <c r="AC13" t="inlineStr">
         <is>
           <t>Conforme</t>
@@ -6576,7 +8018,6 @@
       <c r="W33" t="n">
         <v>2</v>
       </c>
-      <c r="X33" t="inlineStr"/>
       <c r="Y33" t="inlineStr">
         <is>
           <t>Normal</t>
@@ -6587,8 +8028,6 @@
           <t>2025-06-22</t>
         </is>
       </c>
-      <c r="AA33" t="inlineStr"/>
-      <c r="AB33" t="inlineStr"/>
       <c r="AC33" t="inlineStr">
         <is>
           <t>Conforme</t>
@@ -7734,7 +9173,6 @@
       <c r="W41" t="n">
         <v>1</v>
       </c>
-      <c r="X41" t="inlineStr"/>
       <c r="Y41" t="inlineStr">
         <is>
           <t>Normal</t>
@@ -7745,8 +9183,6 @@
           <t>2025-06-22</t>
         </is>
       </c>
-      <c r="AA41" t="inlineStr"/>
-      <c r="AB41" t="inlineStr"/>
       <c r="AC41" t="inlineStr">
         <is>
           <t>Conforme</t>
@@ -7870,7 +9306,6 @@
       <c r="W42" t="n">
         <v>9</v>
       </c>
-      <c r="X42" t="inlineStr"/>
       <c r="Y42" t="inlineStr">
         <is>
           <t>Normal</t>
@@ -7881,8 +9316,6 @@
           <t>2025-06-22</t>
         </is>
       </c>
-      <c r="AA42" t="inlineStr"/>
-      <c r="AB42" t="inlineStr"/>
       <c r="AC42" t="inlineStr">
         <is>
           <t>Conforme</t>
@@ -8590,7 +10023,6 @@
       <c r="W47" t="n">
         <v>2</v>
       </c>
-      <c r="X47" t="inlineStr"/>
       <c r="Y47" t="inlineStr">
         <is>
           <t>Normal</t>
@@ -8601,8 +10033,6 @@
           <t>2025-06-22</t>
         </is>
       </c>
-      <c r="AA47" t="inlineStr"/>
-      <c r="AB47" t="inlineStr"/>
       <c r="AC47" t="inlineStr">
         <is>
           <t>Conforme</t>
@@ -8887,8 +10317,6 @@
           <t>2025-06-22</t>
         </is>
       </c>
-      <c r="AA49" t="inlineStr"/>
-      <c r="AB49" t="inlineStr"/>
       <c r="AC49" t="inlineStr">
         <is>
           <t>Conforme</t>
@@ -9012,7 +10440,6 @@
       <c r="W50" t="n">
         <v>1</v>
       </c>
-      <c r="X50" t="inlineStr"/>
       <c r="Y50" t="inlineStr">
         <is>
           <t>Normal</t>
@@ -9023,8 +10450,6 @@
           <t>2025-06-22</t>
         </is>
       </c>
-      <c r="AA50" t="inlineStr"/>
-      <c r="AB50" t="inlineStr"/>
       <c r="AC50" t="inlineStr">
         <is>
           <t>Conforme</t>
@@ -9148,7 +10573,6 @@
       <c r="W51" t="n">
         <v>7</v>
       </c>
-      <c r="X51" t="inlineStr"/>
       <c r="Y51" t="inlineStr">
         <is>
           <t>Normal</t>
@@ -9159,8 +10583,6 @@
           <t>2025-06-22</t>
         </is>
       </c>
-      <c r="AA51" t="inlineStr"/>
-      <c r="AB51" t="inlineStr"/>
       <c r="AC51" t="inlineStr">
         <is>
           <t>Conforme</t>
@@ -13467,7 +14889,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -13538,7 +14959,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -13609,7 +15029,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -13680,7 +15099,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -13751,7 +15169,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -13822,7 +15239,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -13893,7 +15309,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -13964,7 +15379,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -14035,7 +15449,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -14106,7 +15519,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -14177,7 +15589,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -14248,7 +15659,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -14319,7 +15729,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -14390,7 +15799,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -14461,7 +15869,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -14532,7 +15939,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -14603,7 +16009,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -14674,7 +16079,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -14745,7 +16149,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -14816,7 +16219,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -14887,7 +16289,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -14958,7 +16359,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -15029,7 +16429,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -15100,7 +16499,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -15171,7 +16569,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -15242,7 +16639,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -15313,7 +16709,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -15384,7 +16779,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -15455,7 +16849,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -15526,7 +16919,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -15597,7 +16989,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -15668,7 +17059,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -15739,7 +17129,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -15810,7 +17199,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -15881,7 +17269,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -15952,7 +17339,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -16023,7 +17409,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -16094,7 +17479,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -16165,7 +17549,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -16236,7 +17619,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -16307,7 +17689,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -16378,7 +17759,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -16449,7 +17829,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -16520,7 +17899,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -16591,7 +17969,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -16662,7 +18039,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -16733,7 +18109,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -16804,7 +18179,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -16875,7 +18249,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -16946,7 +18319,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -17017,7 +18389,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -17088,7 +18459,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -17159,7 +18529,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -17230,7 +18599,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -17301,7 +18669,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -17372,7 +18739,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -17443,7 +18809,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -17514,7 +18879,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -17585,7 +18949,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -17656,7 +19019,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -17727,7 +19089,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -17798,7 +19159,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -17869,7 +19229,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -17940,7 +19299,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -18011,7 +19369,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -18082,7 +19439,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -18153,7 +19509,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -18224,7 +19579,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -18295,7 +19649,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -18366,7 +19719,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -18437,7 +19789,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -18508,7 +19859,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -18579,7 +19929,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -18650,7 +19999,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -18721,7 +20069,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -18792,7 +20139,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -18863,7 +20209,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -18934,7 +20279,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -19005,7 +20349,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -19076,7 +20419,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -19147,7 +20489,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -19218,7 +20559,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -19289,7 +20629,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -19360,7 +20699,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -19431,7 +20769,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -19502,7 +20839,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -19573,7 +20909,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -19644,7 +20979,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -19715,7 +21049,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -19786,7 +21119,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -19857,7 +21189,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -19928,7 +21259,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -19999,7 +21329,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -20070,7 +21399,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -20141,7 +21469,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -20212,7 +21539,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -20283,7 +21609,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -20354,7 +21679,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -20425,7 +21749,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -20496,7 +21819,6 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="O101" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -28331,7 +29653,6 @@
           <t>Neutral</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -28414,7 +29735,6 @@
           <t>Positiva</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -28497,7 +29817,6 @@
           <t>Neutral</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -28580,7 +29899,6 @@
           <t>Neutral</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -28663,7 +29981,6 @@
           <t>Neutral</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -28746,7 +30063,6 @@
           <t>Neutral</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -28829,7 +30145,6 @@
           <t>Negativa</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -28912,7 +30227,6 @@
           <t>Neutral</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -28995,7 +30309,6 @@
           <t>Positiva</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -29078,7 +30391,6 @@
           <t>Neutral</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -29161,7 +30473,6 @@
           <t>Neutral</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -29244,7 +30555,6 @@
           <t>Neutral</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -29327,7 +30637,6 @@
           <t>Neutral</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -29410,7 +30719,6 @@
           <t>Neutral</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -29493,7 +30801,6 @@
           <t>Neutral</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -29576,7 +30883,6 @@
           <t>Negativa</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -29659,7 +30965,6 @@
           <t>Positiva</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -29742,7 +31047,6 @@
           <t>Negativa</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -29825,7 +31129,6 @@
           <t>Positiva</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -29908,7 +31211,6 @@
           <t>Negativa</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -29991,7 +31293,6 @@
           <t>Negativa</t>
         </is>
       </c>
-      <c r="S22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -30074,7 +31375,6 @@
           <t>Negativa</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -30157,7 +31457,6 @@
           <t>Negativa</t>
         </is>
       </c>
-      <c r="S24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -30240,7 +31539,6 @@
           <t>Neutral</t>
         </is>
       </c>
-      <c r="S25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -30323,7 +31621,6 @@
           <t>Neutral</t>
         </is>
       </c>
-      <c r="S26" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>